<commit_message>
refactor: Change 'ratios' to 'ratio' in RatioFormula model and related components
</commit_message>
<xml_diff>
--- a/public/sample_uploads/ratio_formulas.xlsx
+++ b/public/sample_uploads/ratio_formulas.xlsx
@@ -327,16 +327,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="5.5" min="1" max="1" bestFit="1" customWidth="1"/>
-    <col width="15.400000000000002" min="2" max="2" bestFit="1" customWidth="1"/>
+    <col width="7.700000000000001" min="2" max="2" bestFit="1" customWidth="1"/>
     <col width="8.8" min="3" max="3" bestFit="1" customWidth="1"/>
     <col width="19.8" min="4" max="4" bestFit="1" customWidth="1"/>
     <col width="9.9" min="5" max="5" bestFit="1" customWidth="1"/>
-    <col width="19.8" min="6" max="6" bestFit="1" customWidth="1"/>
+    <col width="8.8" min="6" max="6" bestFit="1" customWidth="1"/>
     <col width="30.800000000000004" min="7" max="7" bestFit="1" customWidth="1"/>
+    <col width="15.400000000000002" min="8" max="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -347,46 +348,43 @@
       </c>
       <c r="B1" s="0" t="inlineStr">
         <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>Account Entry Names</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
           <t>Update Only</t>
-        </is>
-      </c>
-      <c r="C1" s="0" t="inlineStr">
-        <is>
-          <t>Level</t>
-        </is>
-      </c>
-      <c r="D1" s="0" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="E1" s="0" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="F1" s="0" t="inlineStr">
-        <is>
-          <t>Ratios</t>
-        </is>
-      </c>
-      <c r="G1" s="0" t="inlineStr">
-        <is>
-          <t>Account Entry Names</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="A2" s="0"/>
+      <c r="B2" s="0"/>
       <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Fund</t>
@@ -404,7 +402,7 @@
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
-          <t>XIRR, DPI, TVPI</t>
+          <t>XIRR</t>
         </is>
       </c>
       <c r="G2" s="0" t="inlineStr">
@@ -412,18 +410,11 @@
           <t>Operating Income, Revenue</t>
         </is>
       </c>
+      <c r="H2" s="0"/>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="A3" s="0"/>
+      <c r="B3" s="0"/>
       <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Folio</t>
@@ -441,7 +432,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>MOIC, RVPI</t>
+          <t>MOIC</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
@@ -449,6 +440,7 @@
           <t>Capital Expenditure</t>
         </is>
       </c>
+      <c r="H3" s="0"/>
     </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="1"/>

</xml_diff>